<commit_message>
added jsons for 36_South_China_Sea for northern part from paper 2007 (2 models: 1970s and 2000s)
</commit_message>
<xml_diff>
--- a/13_Humboldt_Current/13_north_(2018)/13_north_(2018)_extracted/13_11013_Humboldt_Current_(1995-2004)_reconstructed.xlsx
+++ b/13_Humboldt_Current/13_north_(2018)/13_north_(2018)_extracted/13_11013_Humboldt_Current_(1995-2004)_reconstructed.xlsx
@@ -7567,22 +7567,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Benthic detritus</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pelagic detritus</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Fishery offal</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Anchovy eggs</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Fishery offal</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Pelagic detritus</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Benthic detritus</t>
         </is>
       </c>
     </row>
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -7625,10 +7625,10 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -7649,10 +7649,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -7670,16 +7670,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -7694,16 +7694,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -7718,16 +7718,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="E7" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -7742,16 +7742,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="E8" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -7766,7 +7766,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -7775,7 +7775,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -7790,7 +7790,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -7799,7 +7799,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -7814,16 +7814,16 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
         <v>0.25</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.75</v>
       </c>
     </row>
     <row r="12">
@@ -7838,16 +7838,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E12" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -7862,7 +7862,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -7871,7 +7871,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E14" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -7910,16 +7910,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E15" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -7934,7 +7934,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -7943,7 +7943,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -7958,7 +7958,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -7967,7 +7967,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -7982,7 +7982,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -7991,7 +7991,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -8006,16 +8006,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -8030,7 +8030,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -8039,7 +8039,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -8054,7 +8054,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -8063,7 +8063,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -8078,16 +8078,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E22" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -8102,16 +8102,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E23" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -8126,7 +8126,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -8135,7 +8135,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -8150,7 +8150,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -8159,7 +8159,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -8174,7 +8174,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -8183,7 +8183,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -8198,7 +8198,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -8207,7 +8207,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -8222,7 +8222,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -8231,7 +8231,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -8246,7 +8246,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -8255,7 +8255,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -8270,7 +8270,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -8279,7 +8279,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -8294,7 +8294,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -8303,7 +8303,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -8318,7 +8318,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -8327,7 +8327,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -8342,7 +8342,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -8351,7 +8351,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -8366,7 +8366,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -8390,16 +8390,16 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="E35" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -8414,16 +8414,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="E36" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -8438,7 +8438,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -8447,7 +8447,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -8462,16 +8462,16 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -8486,7 +8486,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -8495,7 +8495,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
run on all jsons again after fix
</commit_message>
<xml_diff>
--- a/13_Humboldt_Current/13_north_(2018)/13_north_(2018)_extracted/13_11013_Humboldt_Current_(1995-2004)_reconstructed.xlsx
+++ b/13_Humboldt_Current/13_north_(2018)/13_north_(2018)_extracted/13_11013_Humboldt_Current_(1995-2004)_reconstructed.xlsx
@@ -7567,22 +7567,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Pelagic detritus</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fishery offal</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Anchovy eggs</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Benthic detritus</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Pelagic detritus</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Fishery offal</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Anchovy eggs</t>
         </is>
       </c>
     </row>
@@ -7598,10 +7598,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -7622,10 +7622,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -7646,10 +7646,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -7670,16 +7670,16 @@
         </is>
       </c>
       <c r="C5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
         <v>0.8</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -7694,16 +7694,16 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
         <v>0.8</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -7718,16 +7718,16 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
         <v>0.05</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -7742,16 +7742,16 @@
         </is>
       </c>
       <c r="C8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
         <v>0.05</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -7766,7 +7766,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -7775,7 +7775,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -7790,7 +7790,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -7799,7 +7799,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -7814,16 +7814,16 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F11" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.25</v>
       </c>
     </row>
     <row r="12">
@@ -7838,16 +7838,16 @@
         </is>
       </c>
       <c r="C12" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -7862,7 +7862,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -7871,7 +7871,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="C14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -7910,16 +7910,16 @@
         </is>
       </c>
       <c r="C15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -7934,7 +7934,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -7943,7 +7943,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -7958,7 +7958,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -7967,7 +7967,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -7982,7 +7982,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -7991,7 +7991,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -8006,16 +8006,16 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
         <v>0.9</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -8030,7 +8030,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -8039,7 +8039,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -8054,7 +8054,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -8063,7 +8063,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -8078,16 +8078,16 @@
         </is>
       </c>
       <c r="C22" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -8102,16 +8102,16 @@
         </is>
       </c>
       <c r="C23" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -8126,7 +8126,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -8135,7 +8135,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -8150,7 +8150,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -8159,7 +8159,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -8174,7 +8174,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -8183,7 +8183,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -8198,7 +8198,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -8207,7 +8207,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -8222,7 +8222,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -8231,7 +8231,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -8246,7 +8246,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -8255,7 +8255,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -8270,7 +8270,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -8279,7 +8279,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -8294,7 +8294,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
@@ -8303,7 +8303,7 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -8318,7 +8318,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -8327,7 +8327,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -8342,7 +8342,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -8351,7 +8351,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -8366,7 +8366,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -8375,7 +8375,7 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -8390,16 +8390,16 @@
         </is>
       </c>
       <c r="C35" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
         <v>0.3</v>
-      </c>
-      <c r="D35" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -8414,16 +8414,16 @@
         </is>
       </c>
       <c r="C36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
         <v>0.3</v>
-      </c>
-      <c r="D36" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -8438,7 +8438,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
@@ -8447,7 +8447,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -8462,16 +8462,16 @@
         </is>
       </c>
       <c r="C38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
         <v>0.9</v>
-      </c>
-      <c r="D38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -8486,7 +8486,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -8495,7 +8495,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">

</xml_diff>